<commit_message>
Update Checklist to Release Repo_v2025_11_06.xlsx
</commit_message>
<xml_diff>
--- a/Documents/Checklist to Release Repo_v2025_11_06.xlsx
+++ b/Documents/Checklist to Release Repo_v2025_11_06.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D6D4D0-6A44-441A-BDFF-88FF58A000A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ABB229C-EC9E-4C71-A5B2-27287E70F9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -933,7 +933,7 @@
       <c r="D3" s="6"/>
       <c r="E3" s="7"/>
     </row>
-    <row r="4" spans="2:5" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:5" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1192,9 +1192,7 @@
         <v>28</v>
       </c>
       <c r="C26" s="12"/>
-      <c r="D26" s="16">
-        <v>45967</v>
-      </c>
+      <c r="D26" s="16"/>
       <c r="E26" s="13"/>
     </row>
     <row r="27" spans="2:5" ht="69.75" x14ac:dyDescent="0.2">
@@ -1556,30 +1554,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="542b8847-f5d4-4c9f-bd30-657d16e5db1d" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf" xsi:nil="true"/>
-    <Size xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf" xsi:nil="true"/>
-    <Notes xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009204A49901785041AF741C157FF60EBA" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="92f33ed966115dd153c36d444c727f64">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c7c738f6-68ec-422e-b0e4-3523873f7adf" xmlns:ns3="542b8847-f5d4-4c9f-bd30-657d16e5db1d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="af9e6b9a599ebdef525a94f01cc358a4" ns2:_="" ns3:_="">
     <xsd:import namespace="c7c738f6-68ec-422e-b0e4-3523873f7adf"/>
@@ -1860,26 +1834,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4994F8E-3141-47F3-91B7-8A348AFEAE97}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="542b8847-f5d4-4c9f-bd30-657d16e5db1d" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf" xsi:nil="true"/>
+    <Size xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf" xsi:nil="true"/>
+    <Notes xmlns="c7c738f6-68ec-422e-b0e4-3523873f7adf" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B3E0A64-3B79-40D0-B5B8-9F6FE2202932}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="542b8847-f5d4-4c9f-bd30-657d16e5db1d"/>
-    <ds:schemaRef ds:uri="c7c738f6-68ec-422e-b0e4-3523873f7adf"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7756634-8DAD-4D78-BE4D-E15218DE2524}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1898,6 +1877,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B3E0A64-3B79-40D0-B5B8-9F6FE2202932}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="542b8847-f5d4-4c9f-bd30-657d16e5db1d"/>
+    <ds:schemaRef ds:uri="c7c738f6-68ec-422e-b0e4-3523873f7adf"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4994F8E-3141-47F3-91B7-8A348AFEAE97}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{7cf48d45-3ddb-4389-a9c1-c115526eb52e}" enabled="0" method="" siteId="{7cf48d45-3ddb-4389-a9c1-c115526eb52e}" removed="1"/>

</xml_diff>